<commit_message>
Add 2026-10-11 option chains and options sleeve outputs
- IBKR option chains for 11 underlyings (154 contracts, Friday close quotes)
- Rank ideas by return at a one-standard-deviation favourable move weighted
  by probability of profit, so long options are not scored on tail moves
- Options page, brief section and workbook Options sheet regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5kBEyRs7ygwcTxDxKNeBy
</commit_message>
<xml_diff>
--- a/reports/2026-10-11/decision-book.xlsx
+++ b/reports/2026-10-11/decision-book.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Decisions" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="SG Income" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="FX" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Decision Log" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Options" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Decision Log" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$1:$S$84</definedName>
@@ -49,7 +50,7 @@
 </comments>
 </file>
 
-<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
@@ -72,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="406">
   <si>
     <t xml:space="preserve">Global Investment Decision Book</t>
   </si>
@@ -170,6 +171,18 @@
     <t xml:space="preserve">Singapore income target: upper bound</t>
   </si>
   <si>
+    <t xml:space="preserve">Options sleeve cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total option premium at risk, share of portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Options per-trade risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium at risk per option trade</t>
+  </si>
+  <si>
     <t xml:space="preserve">Portfolio tilts this week</t>
   </si>
   <si>
@@ -1110,6 +1123,135 @@
   </si>
   <si>
     <t xml:space="preserve">USD strengthening vs CHF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Underlying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debit / share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Move to breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max gain / share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reward : risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prob. of profit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contracts (per-trade budget)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium at risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stop: close at value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bull call spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 170C / Sell 185C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-12-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bear put spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 385P / Sell 345P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 350C / Sell 385C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 335C / Sell 370C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 140P / Sell 125P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 230C / Sell 250C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 751C / Sell 825C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 779C / Sell 855C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long put</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 135P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 175C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 240C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 370C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 365P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 355C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 789C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 817C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sleeve check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total if all taken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sleeve cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within cap?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability of profit is risk-neutral, from the option's implied volatility. Debits are mid prices from IBKR weekend quotes; re-price live before trading. Defined risk only: maximum loss = premium paid.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -1155,7 +1297,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
@@ -1166,6 +1308,8 @@
     <numFmt numFmtId="171" formatCode="0.000"/>
     <numFmt numFmtId="172" formatCode="0.0000"/>
     <numFmt numFmtId="173" formatCode="0.00%"/>
+    <numFmt numFmtId="174" formatCode="0.0\x"/>
+    <numFmt numFmtId="175" formatCode="General"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1340,7 +1484,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1459,6 +1603,34 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1869,7 +2041,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1976,24 +2148,30 @@
         <v>31</v>
       </c>
     </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>34</v>
       </c>
+      <c r="B11" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="A13" s="9" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2035,6 +2213,22 @@
       </c>
       <c r="C18" s="2" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2075,84 +2269,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H2" s="13" t="n">
         <v>65.08</v>
@@ -2195,25 +2389,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="E3" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="G3" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="H3" s="13" t="n">
         <v>37.954</v>
@@ -2256,25 +2450,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E4" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="H4" s="13" t="n">
         <v>168.94</v>
@@ -2317,25 +2511,25 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H5" s="13" t="n">
         <v>40.31</v>
@@ -2378,25 +2572,25 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H6" s="13" t="n">
         <v>198.78</v>
@@ -2439,25 +2633,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H7" s="13" t="n">
         <v>778.57</v>
@@ -2500,25 +2694,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E8" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="H8" s="13" t="n">
         <v>336.64</v>
@@ -2561,25 +2755,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H9" s="13" t="n">
         <v>751.27</v>
@@ -2622,25 +2816,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H10" s="13" t="n">
         <v>170.81</v>
@@ -2683,25 +2877,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="H11" s="13" t="n">
         <v>351.66</v>
@@ -2744,25 +2938,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E12" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="H12" s="13" t="n">
         <v>229.28</v>
@@ -2805,25 +2999,25 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H13" s="13" t="n">
         <v>275.04</v>
@@ -2866,25 +3060,25 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D14" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>107</v>
-      </c>
       <c r="G14" s="12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H14" s="13" t="n">
         <v>148.2</v>
@@ -2927,25 +3121,25 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H15" s="13" t="n">
         <v>559.4</v>
@@ -2988,25 +3182,25 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H16" s="13" t="n">
         <v>418.78</v>
@@ -3049,25 +3243,25 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H17" s="13" t="n">
         <v>535.07</v>
@@ -3110,25 +3304,25 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="H18" s="13" t="n">
         <v>216.74</v>
@@ -3171,25 +3365,25 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H19" s="13" t="n">
         <v>41.42</v>
@@ -3232,25 +3426,25 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H20" s="13" t="n">
         <v>262.43</v>
@@ -3293,25 +3487,25 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="H21" s="13" t="n">
         <v>112.67</v>
@@ -3354,25 +3548,25 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H22" s="13" t="n">
         <v>28.99</v>
@@ -3415,25 +3609,25 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H23" s="13" t="n">
         <v>718.67</v>
@@ -3476,25 +3670,25 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H24" s="13" t="n">
         <v>140.86</v>
@@ -3537,25 +3731,25 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H25" s="13" t="n">
         <v>27.22</v>
@@ -3598,25 +3792,25 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H26" s="13" t="n">
         <v>46.77</v>
@@ -3659,25 +3853,25 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F27" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H27" s="13" t="n">
         <v>29</v>
@@ -3716,25 +3910,25 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="C28" s="10" t="s">
-        <v>152</v>
-      </c>
       <c r="D28" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F28" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H28" s="13" t="n">
         <v>73.36</v>
@@ -3773,25 +3967,25 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="G29" s="12" t="s">
         <v>158</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F29" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="G29" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="H29" s="13" t="n">
         <v>5.497</v>
@@ -3830,25 +4024,25 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H30" s="13" t="n">
         <v>71.16</v>
@@ -3887,25 +4081,25 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F31" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H31" s="13" t="n">
         <v>13.958</v>
@@ -3944,25 +4138,25 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F32" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H32" s="13" t="n">
         <v>9.83</v>
@@ -4001,25 +4195,25 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H33" s="13" t="n">
         <v>145.2</v>
@@ -4058,25 +4252,25 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H34" s="13" t="n">
         <v>24.53</v>
@@ -4115,25 +4309,25 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H35" s="13" t="n">
         <v>82.46</v>
@@ -4172,25 +4366,25 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H36" s="13" t="n">
         <v>28.33</v>
@@ -4229,25 +4423,25 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H37" s="13" t="n">
         <v>10.266</v>
@@ -4286,25 +4480,25 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H38" s="13" t="n">
         <v>10.42</v>
@@ -4343,25 +4537,25 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H39" s="13" t="n">
         <v>49.43</v>
@@ -4400,25 +4594,25 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H40" s="13" t="n">
         <v>13.844</v>
@@ -4457,25 +4651,25 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H41" s="13" t="n">
         <v>1.016</v>
@@ -4514,25 +4708,25 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H42" s="13" t="n">
         <v>332.99</v>
@@ -4571,25 +4765,25 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H43" s="13" t="n">
         <v>169.25</v>
@@ -4628,25 +4822,25 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F44" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H44" s="13" t="n">
         <v>54.73</v>
@@ -4685,25 +4879,25 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F45" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H45" s="13" t="n">
         <v>39.96</v>
@@ -4742,25 +4936,25 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F46" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H46" s="13" t="n">
         <v>361.54</v>
@@ -4799,25 +4993,25 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F47" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H47" s="13" t="n">
         <v>4.303</v>
@@ -4856,25 +5050,25 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F48" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H48" s="13" t="n">
         <v>11.01</v>
@@ -4913,25 +5107,25 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H49" s="13" t="n">
         <v>86.84</v>
@@ -4970,25 +5164,25 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H50" s="13" t="n">
         <v>18.574</v>
@@ -5027,25 +5221,25 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F51" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H51" s="13" t="n">
         <v>41.61</v>
@@ -5084,25 +5278,25 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H52" s="13" t="n">
         <v>37.32</v>
@@ -5141,25 +5335,25 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F53" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H53" s="13" t="n">
         <v>120.24</v>
@@ -5198,25 +5392,25 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F54" s="20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G54" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H54" s="13" t="n">
         <v>3.98</v>
@@ -5255,25 +5449,25 @@
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F55" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H55" s="13" t="n">
         <v>83.43</v>
@@ -5312,25 +5506,25 @@
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D56" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F56" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="E56" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F56" s="21" t="s">
-        <v>221</v>
-      </c>
       <c r="G56" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H56" s="13" t="n">
         <v>54.78</v>
@@ -5369,25 +5563,25 @@
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F57" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="G57" s="12" t="s">
         <v>226</v>
-      </c>
-      <c r="B57" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="C57" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F57" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="G57" s="12" t="s">
-        <v>222</v>
       </c>
       <c r="H57" s="13" t="n">
         <v>384.58</v>
@@ -5426,25 +5620,25 @@
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F58" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G58" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H58" s="13" t="n">
         <v>52.83</v>
@@ -5483,25 +5677,25 @@
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F59" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G59" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H59" s="13" t="n">
         <v>17.544</v>
@@ -5540,25 +5734,25 @@
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F60" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H60" s="13" t="n">
         <v>11.48</v>
@@ -5597,25 +5791,25 @@
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="D61" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="B61" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="C61" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>231</v>
-      </c>
       <c r="E61" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F61" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G61" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H61" s="13" t="n">
         <v>71.26</v>
@@ -5654,25 +5848,25 @@
     </row>
     <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F62" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H62" s="13" t="n">
         <v>4.24</v>
@@ -5711,25 +5905,25 @@
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="10" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F63" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G63" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H63" s="13" t="n">
         <v>110.38</v>
@@ -5768,25 +5962,25 @@
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F64" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H64" s="13" t="n">
         <v>0.955</v>
@@ -5825,25 +6019,25 @@
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F65" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G65" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H65" s="13" t="n">
         <v>1263</v>
@@ -5882,25 +6076,25 @@
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F66" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G66" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H66" s="13" t="n">
         <v>80.1</v>
@@ -5939,25 +6133,25 @@
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F67" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G67" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H67" s="13" t="n">
         <v>112.85</v>
@@ -5996,25 +6190,25 @@
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F68" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H68" s="13" t="n">
         <v>24.84</v>
@@ -6053,25 +6247,25 @@
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F69" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G69" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H69" s="13" t="n">
         <v>52.24</v>
@@ -6110,25 +6304,25 @@
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="10" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F70" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H70" s="13" t="n">
         <v>141.4</v>
@@ -6167,25 +6361,25 @@
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="10" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F71" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G71" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H71" s="13" t="n">
         <v>107</v>
@@ -6224,25 +6418,25 @@
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F72" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H72" s="13" t="n">
         <v>377.8</v>
@@ -6281,25 +6475,25 @@
     </row>
     <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B73" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="C73" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="D73" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="C73" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>261</v>
-      </c>
       <c r="E73" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F73" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G73" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H73" s="13" t="n">
         <v>71.5</v>
@@ -6338,25 +6532,25 @@
     </row>
     <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F74" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G74" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H74" s="13" t="n">
         <v>2.24</v>
@@ -6395,25 +6589,25 @@
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F75" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G75" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H75" s="13" t="n">
         <v>41.41</v>
@@ -6452,25 +6646,25 @@
     </row>
     <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F76" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H76" s="13" t="n">
         <v>297.75</v>
@@ -6509,25 +6703,25 @@
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F77" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G77" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H77" s="13" t="n">
         <v>75.6</v>
@@ -6566,25 +6760,25 @@
     </row>
     <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F78" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G78" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H78" s="13" t="n">
         <v>2.13</v>
@@ -6623,25 +6817,25 @@
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F79" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G79" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H79" s="13" t="n">
         <v>424.8</v>
@@ -6680,25 +6874,25 @@
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F80" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H80" s="13" t="n">
         <v>1.08</v>
@@ -6737,25 +6931,25 @@
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F81" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G81" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H81" s="13" t="n">
         <v>1.83</v>
@@ -6794,25 +6988,25 @@
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F82" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G82" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H82" s="13" t="n">
         <v>2.07</v>
@@ -6851,25 +7045,25 @@
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F83" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G83" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H83" s="13" t="n">
         <v>1.19</v>
@@ -6908,25 +7102,25 @@
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F84" s="21" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G84" s="12" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H84" s="13" t="n">
         <v>2.19</v>
@@ -6965,10 +7159,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="9" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="N86" s="9" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="O86" s="22" t="n">
         <f aca="false">SUM(O2:O84)</f>
@@ -6981,7 +7175,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -7020,51 +7214,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C2" s="24" t="n">
         <v>1.83</v>
@@ -7100,18 +7294,18 @@
         <v>-0.144859813084112</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M2" s="29" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C3" s="24" t="n">
         <v>2.19</v>
@@ -7147,18 +7341,18 @@
         <v>-0.22887323943662</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M3" s="29" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>1.08</v>
@@ -7194,18 +7388,18 @@
         <v>-0.142857142857143</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M4" s="29" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C5" s="24" t="n">
         <v>1.19</v>
@@ -7241,18 +7435,18 @@
         <v>-0.179310344827586</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M5" s="29" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>2.13</v>
@@ -7288,18 +7482,18 @@
         <v>-0.108786610878661</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M6" s="29" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>2.07</v>
@@ -7335,18 +7529,18 @@
         <v>-0.130252100840336</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="M7" s="29" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>0.955</v>
@@ -7382,18 +7576,18 @@
         <v>-0.00520833333333337</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="M8" s="29" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>2.24</v>
@@ -7429,18 +7623,18 @@
         <v>-0.0427350427350426</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="M9" s="29" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>4.24</v>
@@ -7476,18 +7670,18 @@
         <v>-0.00469483568075102</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="M10" s="29" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>73.36</v>
@@ -7523,18 +7717,18 @@
         <v>0.36230269266481</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M11" s="29" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>3.98</v>
@@ -7570,18 +7764,18 @@
         <v>-0.038647342995169</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M12" s="29" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>39.96</v>
@@ -7617,18 +7811,18 @@
         <v>0.13105009906595</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M13" s="29" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>29</v>
@@ -7664,18 +7858,18 @@
         <v>0.718009478672986</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M14" s="29" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>10.42</v>
@@ -7711,15 +7905,15 @@
         <v>0.218713450292398</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M15" s="29" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -7749,27 +7943,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D2" s="28" t="n">
         <v>-0.0127528665983034</v>
@@ -7777,13 +7971,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="D3" s="28" t="n">
         <v>-0.0188782549659446</v>
@@ -7791,13 +7985,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="D4" s="28" t="n">
         <v>-0.00660327522451132</v>
@@ -7805,13 +7999,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>-0.0208884147378512</v>
@@ -7819,13 +8013,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D6" s="28" t="n">
         <v>-0.00849671937600405</v>
@@ -7833,13 +8027,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D7" s="28" t="n">
         <v>0.00107789548878423</v>
@@ -7847,13 +8041,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D8" s="28" t="n">
         <v>-0.0131264168678695</v>
@@ -7861,13 +8055,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D9" s="28" t="n">
         <v>0.00377317809400601</v>
@@ -7875,13 +8069,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D10" s="28" t="n">
         <v>0.0268097343764495</v>
@@ -7899,6 +8093,1058 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:Q23"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E2" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F2" s="31" t="n">
+        <v>168.79</v>
+      </c>
+      <c r="G2" s="32" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="H2" s="23" t="n">
+        <f aca="false">G2*100</f>
+        <v>487</v>
+      </c>
+      <c r="I2" s="31" t="n">
+        <v>174.87</v>
+      </c>
+      <c r="J2" s="33" t="n">
+        <f aca="false">I2/F2-1</f>
+        <v>0.0360210912968779</v>
+      </c>
+      <c r="K2" s="32" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="L2" s="34" t="n">
+        <f aca="false">IF(K2="","open",K2/G2)</f>
+        <v>2.08008213552361</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>0.387158488416082</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>0.281044545535459</v>
+      </c>
+      <c r="O2" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H2)</f>
+        <v>20</v>
+      </c>
+      <c r="P2" s="23" t="n">
+        <f aca="false">O2*H2</f>
+        <v>9740</v>
+      </c>
+      <c r="Q2" s="36" t="n">
+        <f aca="false">G2*(1-0.5)</f>
+        <v>2.435</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E3" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F3" s="31" t="n">
+        <v>384.5</v>
+      </c>
+      <c r="G3" s="32" t="n">
+        <v>10.935</v>
+      </c>
+      <c r="H3" s="23" t="n">
+        <f aca="false">G3*100</f>
+        <v>1093.5</v>
+      </c>
+      <c r="I3" s="31" t="n">
+        <v>374.065</v>
+      </c>
+      <c r="J3" s="33" t="n">
+        <f aca="false">I3/F3-1</f>
+        <v>-0.0271391417425227</v>
+      </c>
+      <c r="K3" s="32" t="n">
+        <v>29.065</v>
+      </c>
+      <c r="L3" s="34" t="n">
+        <f aca="false">IF(K3="","open",K3/G3)</f>
+        <v>2.65797896662094</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>0.369628364966556</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>0.211865064588511</v>
+      </c>
+      <c r="O3" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H3)</f>
+        <v>9</v>
+      </c>
+      <c r="P3" s="23" t="n">
+        <f aca="false">O3*H3</f>
+        <v>9841.5</v>
+      </c>
+      <c r="Q3" s="36" t="n">
+        <f aca="false">G3*(1-0.5)</f>
+        <v>5.4675</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F4" s="31" t="n">
+        <v>351.6</v>
+      </c>
+      <c r="G4" s="32" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <f aca="false">G4*100</f>
+        <v>1315</v>
+      </c>
+      <c r="I4" s="31" t="n">
+        <v>363.15</v>
+      </c>
+      <c r="J4" s="33" t="n">
+        <f aca="false">I4/F4-1</f>
+        <v>0.0328498293515358</v>
+      </c>
+      <c r="K4" s="32" t="n">
+        <v>21.85</v>
+      </c>
+      <c r="L4" s="34" t="n">
+        <f aca="false">IF(K4="","open",K4/G4)</f>
+        <v>1.66159695817491</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0.403716166404712</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0.326997925546259</v>
+      </c>
+      <c r="O4" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H4)</f>
+        <v>7</v>
+      </c>
+      <c r="P4" s="23" t="n">
+        <f aca="false">O4*H4</f>
+        <v>9205</v>
+      </c>
+      <c r="Q4" s="36" t="n">
+        <f aca="false">G4*(1-0.5)</f>
+        <v>6.575</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>336.08</v>
+      </c>
+      <c r="G5" s="32" t="n">
+        <v>12.65</v>
+      </c>
+      <c r="H5" s="23" t="n">
+        <f aca="false">G5*100</f>
+        <v>1265</v>
+      </c>
+      <c r="I5" s="31" t="n">
+        <v>347.65</v>
+      </c>
+      <c r="J5" s="33" t="n">
+        <f aca="false">I5/F5-1</f>
+        <v>0.0344263270649845</v>
+      </c>
+      <c r="K5" s="32" t="n">
+        <v>22.35</v>
+      </c>
+      <c r="L5" s="34" t="n">
+        <f aca="false">IF(K5="","open",K5/G5)</f>
+        <v>1.76679841897233</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0.38331306816479</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0.246064122871679</v>
+      </c>
+      <c r="O5" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H5)</f>
+        <v>7</v>
+      </c>
+      <c r="P5" s="23" t="n">
+        <f aca="false">O5*H5</f>
+        <v>8855</v>
+      </c>
+      <c r="Q5" s="36" t="n">
+        <f aca="false">G5*(1-0.5)</f>
+        <v>6.325</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F6" s="31" t="n">
+        <v>141.55</v>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <f aca="false">G6*100</f>
+        <v>655</v>
+      </c>
+      <c r="I6" s="31" t="n">
+        <v>133.45</v>
+      </c>
+      <c r="J6" s="33" t="n">
+        <f aca="false">I6/F6-1</f>
+        <v>-0.0572235959025081</v>
+      </c>
+      <c r="K6" s="32" t="n">
+        <v>8.45</v>
+      </c>
+      <c r="L6" s="34" t="n">
+        <f aca="false">IF(K6="","open",K6/G6)</f>
+        <v>1.29007633587786</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0.443122516868418</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.568444856283021</v>
+      </c>
+      <c r="O6" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H6)</f>
+        <v>15</v>
+      </c>
+      <c r="P6" s="23" t="n">
+        <f aca="false">O6*H6</f>
+        <v>9825</v>
+      </c>
+      <c r="Q6" s="36" t="n">
+        <f aca="false">G6*(1-0.5)</f>
+        <v>3.275</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>229.33</v>
+      </c>
+      <c r="G7" s="32" t="n">
+        <v>7.825</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <f aca="false">G7*100</f>
+        <v>782.5</v>
+      </c>
+      <c r="I7" s="31" t="n">
+        <v>237.825</v>
+      </c>
+      <c r="J7" s="33" t="n">
+        <f aca="false">I7/F7-1</f>
+        <v>0.0370426895739762</v>
+      </c>
+      <c r="K7" s="32" t="n">
+        <v>12.175</v>
+      </c>
+      <c r="L7" s="34" t="n">
+        <f aca="false">IF(K7="","open",K7/G7)</f>
+        <v>1.55591054313099</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0.394779768673195</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>0.340953465060969</v>
+      </c>
+      <c r="O7" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H7)</f>
+        <v>12</v>
+      </c>
+      <c r="P7" s="23" t="n">
+        <f aca="false">O7*H7</f>
+        <v>9390</v>
+      </c>
+      <c r="Q7" s="36" t="n">
+        <f aca="false">G7*(1-0.5)</f>
+        <v>3.9125</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>751.38</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>25.26</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <f aca="false">G8*100</f>
+        <v>2526</v>
+      </c>
+      <c r="I8" s="31" t="n">
+        <v>776.26</v>
+      </c>
+      <c r="J8" s="33" t="n">
+        <f aca="false">I8/F8-1</f>
+        <v>0.0331124065053634</v>
+      </c>
+      <c r="K8" s="32" t="n">
+        <v>48.74</v>
+      </c>
+      <c r="L8" s="34" t="n">
+        <f aca="false">IF(K8="","open",K8/G8)</f>
+        <v>1.92953285827395</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0.368962735908992</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0.194792627653838</v>
+      </c>
+      <c r="O8" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H8)</f>
+        <v>3</v>
+      </c>
+      <c r="P8" s="23" t="n">
+        <f aca="false">O8*H8</f>
+        <v>7578</v>
+      </c>
+      <c r="Q8" s="36" t="n">
+        <f aca="false">G8*(1-0.5)</f>
+        <v>12.63</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>778.57</v>
+      </c>
+      <c r="G9" s="32" t="n">
+        <v>20.395</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <f aca="false">G9*100</f>
+        <v>2039.5</v>
+      </c>
+      <c r="I9" s="31" t="n">
+        <v>799.395</v>
+      </c>
+      <c r="J9" s="33" t="n">
+        <f aca="false">I9/F9-1</f>
+        <v>0.0267477555004687</v>
+      </c>
+      <c r="K9" s="32" t="n">
+        <v>55.605</v>
+      </c>
+      <c r="L9" s="34" t="n">
+        <f aca="false">IF(K9="","open",K9/G9)</f>
+        <v>2.72640353027703</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0.363472788907844</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0.133650255019125</v>
+      </c>
+      <c r="O9" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H9)</f>
+        <v>4</v>
+      </c>
+      <c r="P9" s="23" t="n">
+        <f aca="false">O9*H9</f>
+        <v>8158</v>
+      </c>
+      <c r="Q9" s="36" t="n">
+        <f aca="false">G9*(1-0.5)</f>
+        <v>10.1975</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F10" s="31" t="n">
+        <v>141.55</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <f aca="false">G10*100</f>
+        <v>1015</v>
+      </c>
+      <c r="I10" s="31" t="n">
+        <v>124.85</v>
+      </c>
+      <c r="J10" s="33" t="n">
+        <f aca="false">I10/F10-1</f>
+        <v>-0.117979512539739</v>
+      </c>
+      <c r="K10" s="32"/>
+      <c r="L10" s="34" t="str">
+        <f aca="false">IF(K10="","open",K10/G10)</f>
+        <v>open</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.339881226108832</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>0.566607287616487</v>
+      </c>
+      <c r="O10" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H10)</f>
+        <v>9</v>
+      </c>
+      <c r="P10" s="23" t="n">
+        <f aca="false">O10*H10</f>
+        <v>9135</v>
+      </c>
+      <c r="Q10" s="36" t="n">
+        <f aca="false">G10*(1-0.5)</f>
+        <v>5.075</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>168.79</v>
+      </c>
+      <c r="G11" s="32" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <f aca="false">G11*100</f>
+        <v>565</v>
+      </c>
+      <c r="I11" s="31" t="n">
+        <v>180.65</v>
+      </c>
+      <c r="J11" s="33" t="n">
+        <f aca="false">I11/F11-1</f>
+        <v>0.0702648261152912</v>
+      </c>
+      <c r="K11" s="32"/>
+      <c r="L11" s="34" t="str">
+        <f aca="false">IF(K11="","open",K11/G11)</f>
+        <v>open</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0.289317614247436</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>0.278166458712079</v>
+      </c>
+      <c r="O11" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H11)</f>
+        <v>17</v>
+      </c>
+      <c r="P11" s="23" t="n">
+        <f aca="false">O11*H11</f>
+        <v>9605</v>
+      </c>
+      <c r="Q11" s="36" t="n">
+        <f aca="false">G11*(1-0.5)</f>
+        <v>2.825</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F12" s="31" t="n">
+        <v>229.33</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>9.725</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <f aca="false">G12*100</f>
+        <v>972.5</v>
+      </c>
+      <c r="I12" s="31" t="n">
+        <v>249.725</v>
+      </c>
+      <c r="J12" s="33" t="n">
+        <f aca="false">I12/F12-1</f>
+        <v>0.0889329786770157</v>
+      </c>
+      <c r="K12" s="32"/>
+      <c r="L12" s="34" t="str">
+        <f aca="false">IF(K12="","open",K12/G12)</f>
+        <v>open</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>0.273762735822154</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>0.335245429054431</v>
+      </c>
+      <c r="O12" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H12)</f>
+        <v>10</v>
+      </c>
+      <c r="P12" s="23" t="n">
+        <f aca="false">O12*H12</f>
+        <v>9725</v>
+      </c>
+      <c r="Q12" s="36" t="n">
+        <f aca="false">G12*(1-0.5)</f>
+        <v>4.8625</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F13" s="31" t="n">
+        <v>351.6</v>
+      </c>
+      <c r="G13" s="32" t="n">
+        <v>13.675</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <f aca="false">G13*100</f>
+        <v>1367.5</v>
+      </c>
+      <c r="I13" s="31" t="n">
+        <v>383.675</v>
+      </c>
+      <c r="J13" s="33" t="n">
+        <f aca="false">I13/F13-1</f>
+        <v>0.0912258248009101</v>
+      </c>
+      <c r="K13" s="32"/>
+      <c r="L13" s="34" t="str">
+        <f aca="false">IF(K13="","open",K13/G13)</f>
+        <v>open</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0.263871389642364</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>0.324467860851498</v>
+      </c>
+      <c r="O13" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H13)</f>
+        <v>7</v>
+      </c>
+      <c r="P13" s="23" t="n">
+        <f aca="false">O13*H13</f>
+        <v>9572.5</v>
+      </c>
+      <c r="Q13" s="36" t="n">
+        <f aca="false">G13*(1-0.5)</f>
+        <v>6.8375</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F14" s="31" t="n">
+        <v>384.5</v>
+      </c>
+      <c r="G14" s="32" t="n">
+        <v>5.525</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <f aca="false">G14*100</f>
+        <v>552.5</v>
+      </c>
+      <c r="I14" s="31" t="n">
+        <v>359.475</v>
+      </c>
+      <c r="J14" s="33" t="n">
+        <f aca="false">I14/F14-1</f>
+        <v>-0.0650845253576072</v>
+      </c>
+      <c r="K14" s="32"/>
+      <c r="L14" s="34" t="str">
+        <f aca="false">IF(K14="","open",K14/G14)</f>
+        <v>open</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0.22652457613958</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>0.214702125013975</v>
+      </c>
+      <c r="O14" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H14)</f>
+        <v>18</v>
+      </c>
+      <c r="P14" s="23" t="n">
+        <f aca="false">O14*H14</f>
+        <v>9945</v>
+      </c>
+      <c r="Q14" s="36" t="n">
+        <f aca="false">G14*(1-0.5)</f>
+        <v>2.7625</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F15" s="31" t="n">
+        <v>336.08</v>
+      </c>
+      <c r="G15" s="32" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="H15" s="23" t="n">
+        <f aca="false">G15*100</f>
+        <v>775</v>
+      </c>
+      <c r="I15" s="31" t="n">
+        <v>362.75</v>
+      </c>
+      <c r="J15" s="33" t="n">
+        <f aca="false">I15/F15-1</f>
+        <v>0.0793561056891217</v>
+      </c>
+      <c r="K15" s="32"/>
+      <c r="L15" s="34" t="str">
+        <f aca="false">IF(K15="","open",K15/G15)</f>
+        <v>open</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0.237030626911625</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>0.236173523215233</v>
+      </c>
+      <c r="O15" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H15)</f>
+        <v>12</v>
+      </c>
+      <c r="P15" s="23" t="n">
+        <f aca="false">O15*H15</f>
+        <v>9300</v>
+      </c>
+      <c r="Q15" s="36" t="n">
+        <f aca="false">G15*(1-0.5)</f>
+        <v>3.875</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F16" s="31" t="n">
+        <v>751.38</v>
+      </c>
+      <c r="G16" s="32" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="H16" s="23" t="n">
+        <f aca="false">G16*100</f>
+        <v>1102</v>
+      </c>
+      <c r="I16" s="31" t="n">
+        <v>800.02</v>
+      </c>
+      <c r="J16" s="33" t="n">
+        <f aca="false">I16/F16-1</f>
+        <v>0.0647342223641831</v>
+      </c>
+      <c r="K16" s="32"/>
+      <c r="L16" s="34" t="str">
+        <f aca="false">IF(K16="","open",K16/G16)</f>
+        <v>open</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0.224316324820298</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>0.174740994153321</v>
+      </c>
+      <c r="O16" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H16)</f>
+        <v>9</v>
+      </c>
+      <c r="P16" s="23" t="n">
+        <f aca="false">O16*H16</f>
+        <v>9918</v>
+      </c>
+      <c r="Q16" s="36" t="n">
+        <f aca="false">G16*(1-0.5)</f>
+        <v>5.51</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="F17" s="31" t="n">
+        <v>778.57</v>
+      </c>
+      <c r="G17" s="32" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="H17" s="23" t="n">
+        <f aca="false">G17*100</f>
+        <v>466</v>
+      </c>
+      <c r="I17" s="31" t="n">
+        <v>821.66</v>
+      </c>
+      <c r="J17" s="33" t="n">
+        <f aca="false">I17/F17-1</f>
+        <v>0.0553450556790012</v>
+      </c>
+      <c r="K17" s="32"/>
+      <c r="L17" s="34" t="str">
+        <f aca="false">IF(K17="","open",K17/G17)</f>
+        <v>open</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>0.171791316837144</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <v>0.114405791873116</v>
+      </c>
+      <c r="O17" s="35" t="n">
+        <f aca="false">INT(Policy!$B$2*Policy!$B$11/H17)</f>
+        <v>21</v>
+      </c>
+      <c r="P17" s="23" t="n">
+        <f aca="false">O17*H17</f>
+        <v>9786</v>
+      </c>
+      <c r="Q17" s="36" t="n">
+        <f aca="false">G17*(1-0.5)</f>
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="O19" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="P19" s="23" t="n">
+        <f aca="false">SUM(P2:P17)</f>
+        <v>149579</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O20" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="P20" s="23" t="n">
+        <f aca="false">Policy!$B$2*Policy!$B$10</f>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O21" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="P21" s="0" t="str">
+        <f aca="false">IF(P19&lt;=P20,"Yes","No: pick fewer trades")</f>
+        <v>No: pick fewer trades</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>392</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -7919,71 +9165,71 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>346</v>
+        <v>393</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>347</v>
+        <v>394</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>348</v>
+        <v>395</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>349</v>
+        <v>396</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>350</v>
+        <v>397</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>351</v>
+        <v>398</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>352</v>
+        <v>399</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>353</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
-        <v>354</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="30" t="n">
+      <c r="A2" s="37" t="s">
+        <v>401</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="37" t="n">
         <v>65.08</v>
       </c>
-      <c r="E2" s="31" t="n">
+      <c r="E2" s="38" t="n">
         <v>0.029</v>
       </c>
-      <c r="F2" s="30" t="n">
+      <c r="F2" s="37" t="n">
         <v>55.59</v>
       </c>
-      <c r="G2" s="30" t="s">
-        <v>355</v>
-      </c>
-      <c r="H2" s="30" t="s">
-        <v>356</v>
-      </c>
-      <c r="I2" s="30" t="s">
-        <v>357</v>
-      </c>
-      <c r="J2" s="30" t="s">
-        <v>358</v>
-      </c>
-      <c r="K2" s="30"/>
+      <c r="G2" s="37" t="s">
+        <v>402</v>
+      </c>
+      <c r="H2" s="37" t="s">
+        <v>403</v>
+      </c>
+      <c r="I2" s="37" t="s">
+        <v>404</v>
+      </c>
+      <c r="J2" s="37" t="s">
+        <v>405</v>
+      </c>
+      <c r="K2" s="37"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Revalidation, part 2: full-universe 19-year test, T-bill cash, sustainable SG yields
- weekly_long now covers all 98 instruments by snapshot group (IBKR, verbatim); every
  overlapping week matches the snapshots exactly; rates.json holds the CBOE 13-week T-bill
- backtest on the 83 rated names: Desk process 7.4%/Sharpe 0.62/worst -22.5% vs same
  exposure 7.6%/0.63/-22.9% and always-invested 9.8%/0.69/-44.1%; cluster cap worse again;
  no variant passes adoption; confidence stays LOW
- documented data exceptions (Rolls-Royce rights issue window) and four 2007 unit errors
- SG income decisions use the sustainable yield (lower of 12-month and 4-year average cash
  from IBKR corporate actions); AJBU leaves the band (6.21% -> 4.97%)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5kBEyRs7ygwcTxDxKNeBy
</commit_message>
<xml_diff>
--- a/reports/2026-10-11/decision-book.xlsx
+++ b/reports/2026-10-11/decision-book.xlsx
@@ -1026,34 +1026,34 @@
     <t xml:space="preserve">Yield in target band but price in down-trend: stage in thirds (now, at 1.131 for 7% yield, and after trend repair).</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield in target band but price in down-trend: stage in thirds (now, at 1.889 for 7% yield, and after trend repair).</t>
+    <t xml:space="preserve">Yield 4.97% below band; would reach 6% at 1.765.</t>
   </si>
   <si>
     <t xml:space="preserve">Yield 5.84% below band; would reach 6% at 2.016.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield 5.68% below band; would reach 6% at 0.903.</t>
+    <t xml:space="preserve">Yield 5.58% below band; would reach 6% at 0.888.</t>
   </si>
   <si>
     <t xml:space="preserve">Yield 4.75% below band; would reach 6% at 1.772.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield 4.36% below band; would reach 6% at 3.083.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yield 4.33% below band; would reach 6% at 53.000.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yield 4.12% below band; would reach 6% at 2.735.</t>
+    <t xml:space="preserve">Yield 3.86% below band; would reach 6% at 2.725.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yield 3.44% below band; would reach 6% at 42.083.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yield 3.84% below band; would reach 6% at 2.545.</t>
   </si>
   <si>
     <t xml:space="preserve">Yield 3.98% below band; would reach 6% at 26.500.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield 3.62% below band; would reach 6% at 17.500.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yield 2.30% below band; would reach 6% at 4.000.</t>
+    <t xml:space="preserve">Yield 3.18% below band; would reach 6% at 15.375.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yield 1.75% below band; would reach 6% at 3.042.</t>
   </si>
   <si>
     <t xml:space="preserve">Trailing cash = distributions with ex-date in the 365 days to the as-of date, from IBKR corporate actions, cross-checked to IBKR dividend yield.</t>
@@ -7441,7 +7441,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>281</v>
       </c>
@@ -7482,7 +7482,7 @@
         <v>-0.108786610878661</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>75</v>
+        <v>225</v>
       </c>
       <c r="M6" s="29" t="s">
         <v>317</v>

</xml_diff>